<commit_message>
Move os dois Plexus para a categoria Espumante
Ajuste feito na planilha: Plexus Espumante Branco (era Branco) e Plexus
Espumante Rosé (era Rosé) passam a aparecer na aba Espumante, que agora tem 3
vinhos. Planilha atualizada junto. Cache do service worker v12 -> v13.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Produto_Todos_Vinhos.xlsx
+++ b/Planilha_Produto_Todos_Vinhos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f88f9e9a0b886b5b/Nova_Vinho_Harmonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C57115-7EBD-4194-AE9A-8E63635E7675}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F02A2EAB-7882-4827-A1EA-6D7C8C307BE7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="367">
   <si>
     <t>Nome Vinho</t>
   </si>
@@ -814,9 +814,6 @@
   </si>
   <si>
     <t>Plexus Espumante Rosé</t>
-  </si>
-  <si>
-    <t>Róse</t>
   </si>
   <si>
     <t>Pode Ser</t>
@@ -1624,7 +1621,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -2861,7 +2858,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="67.2" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:12" ht="84" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>136</v>
       </c>
@@ -3279,7 +3276,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>170</v>
       </c>
@@ -3583,7 +3580,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>200</v>
       </c>
@@ -3685,13 +3682,13 @@
         <v>15</v>
       </c>
       <c r="I55" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="J55" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="J55" s="11" t="s">
+      <c r="K55" s="11" t="s">
         <v>282</v>
-      </c>
-      <c r="K55" s="11" t="s">
-        <v>283</v>
       </c>
       <c r="L55" s="11" t="s">
         <v>199</v>
@@ -3723,7 +3720,7 @@
         <v>32</v>
       </c>
       <c r="I56" s="15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J56" s="11" t="s">
         <v>17</v>
@@ -3758,10 +3755,10 @@
         <v>0.115</v>
       </c>
       <c r="H57" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I57" s="15" t="s">
         <v>285</v>
-      </c>
-      <c r="I57" s="15" t="s">
-        <v>286</v>
       </c>
       <c r="J57" s="11" t="s">
         <v>24</v>
@@ -3796,10 +3793,10 @@
         <v>0.14499999999999999</v>
       </c>
       <c r="H58" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="I58" s="15" t="s">
         <v>287</v>
-      </c>
-      <c r="I58" s="15" t="s">
-        <v>288</v>
       </c>
       <c r="J58" s="11" t="s">
         <v>17</v>
@@ -3834,10 +3831,10 @@
         <v>0.13</v>
       </c>
       <c r="H59" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="I59" s="15" t="s">
         <v>289</v>
-      </c>
-      <c r="I59" s="15" t="s">
-        <v>290</v>
       </c>
       <c r="J59" s="11" t="s">
         <v>17</v>
@@ -3872,10 +3869,10 @@
         <v>0.125</v>
       </c>
       <c r="H60" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="I60" s="15" t="s">
         <v>291</v>
-      </c>
-      <c r="I60" s="15" t="s">
-        <v>292</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>24</v>
@@ -3884,7 +3881,7 @@
         <v>43</v>
       </c>
       <c r="L60" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3913,7 +3910,7 @@
         <v>47</v>
       </c>
       <c r="I61" s="15" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J61" s="11" t="s">
         <v>17</v>
@@ -3951,7 +3948,7 @@
         <v>47</v>
       </c>
       <c r="I62" s="15" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J62" s="11" t="s">
         <v>26</v>
@@ -3989,7 +3986,7 @@
         <v>47</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>17</v>
@@ -4027,13 +4024,13 @@
         <v>32</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J64" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="K64" s="11" t="s">
         <v>282</v>
-      </c>
-      <c r="K64" s="11" t="s">
-        <v>283</v>
       </c>
       <c r="L64" s="11" t="s">
         <v>199</v>
@@ -4062,13 +4059,13 @@
         <v>0.13</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I65" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="J65" s="11" t="s">
         <v>298</v>
-      </c>
-      <c r="J65" s="11" t="s">
-        <v>299</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>18</v>
@@ -4100,10 +4097,10 @@
         <v>0.13</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I66" s="15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J66" s="11" t="s">
         <v>17</v>
@@ -4138,10 +4135,10 @@
         <v>0.13</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I67" s="15" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J67" s="11" t="s">
         <v>17</v>
@@ -4176,16 +4173,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H68" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="I68" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="I68" s="15" t="s">
+      <c r="J68" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K68" s="11" t="s">
         <v>303</v>
-      </c>
-      <c r="J68" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K68" s="11" t="s">
-        <v>304</v>
       </c>
       <c r="L68" s="11" t="s">
         <v>82</v>
@@ -4214,10 +4211,10 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H69" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="I69" s="15" t="s">
         <v>305</v>
-      </c>
-      <c r="I69" s="15" t="s">
-        <v>306</v>
       </c>
       <c r="J69" s="11" t="s">
         <v>17</v>
@@ -4252,10 +4249,10 @@
         <v>0.13</v>
       </c>
       <c r="H70" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="I70" s="15" t="s">
         <v>307</v>
-      </c>
-      <c r="I70" s="15" t="s">
-        <v>308</v>
       </c>
       <c r="J70" s="11" t="s">
         <v>17</v>
@@ -4290,10 +4287,10 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H71" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J71" s="11" t="s">
         <v>17</v>
@@ -4331,7 +4328,7 @@
         <v>41</v>
       </c>
       <c r="I72" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>17</v>
@@ -4366,10 +4363,10 @@
         <v>0.13</v>
       </c>
       <c r="H73" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="I73" s="15" t="s">
         <v>311</v>
-      </c>
-      <c r="I73" s="15" t="s">
-        <v>312</v>
       </c>
       <c r="J73" s="11" t="s">
         <v>18</v>
@@ -4404,10 +4401,10 @@
         <v>0.11</v>
       </c>
       <c r="H74" s="11" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I74" s="15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J74" s="11" t="s">
         <v>24</v>
@@ -4445,10 +4442,10 @@
         <v>47</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K75" s="11" t="s">
         <v>18</v>
@@ -4483,7 +4480,7 @@
         <v>47</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>17</v>
@@ -4521,7 +4518,7 @@
         <v>47</v>
       </c>
       <c r="I77" s="15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J77" s="11" t="s">
         <v>17</v>
@@ -4559,7 +4556,7 @@
         <v>47</v>
       </c>
       <c r="I78" s="15" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J78" s="11" t="s">
         <v>17</v>
@@ -4594,10 +4591,10 @@
         <v>0.127</v>
       </c>
       <c r="H79" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="I79" s="15" t="s">
         <v>318</v>
-      </c>
-      <c r="I79" s="15" t="s">
-        <v>319</v>
       </c>
       <c r="J79" s="11" t="s">
         <v>17</v>
@@ -4632,16 +4629,16 @@
         <v>0.125</v>
       </c>
       <c r="H80" s="11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I80" s="15" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J80" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K80" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L80" s="11" t="s">
         <v>82</v>
@@ -4673,13 +4670,13 @@
         <v>47</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J81" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="K81" s="11" t="s">
         <v>282</v>
-      </c>
-      <c r="K81" s="11" t="s">
-        <v>283</v>
       </c>
       <c r="L81" s="11" t="s">
         <v>199</v>
@@ -4708,10 +4705,10 @@
         <v>0.12</v>
       </c>
       <c r="H82" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J82" s="11" t="s">
         <v>26</v>
@@ -4728,7 +4725,7 @@
         <v>239</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>40</v>
+        <v>119</v>
       </c>
       <c r="C83" s="7">
         <v>43.932000000000002</v>
@@ -4749,7 +4746,7 @@
         <v>22</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J83" s="11" t="s">
         <v>26</v>
@@ -4766,7 +4763,7 @@
         <v>240</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>241</v>
+        <v>119</v>
       </c>
       <c r="C84" s="7">
         <v>43.932000000000002</v>
@@ -4787,7 +4784,7 @@
         <v>22</v>
       </c>
       <c r="I84" s="15" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="J84" s="11" t="s">
         <v>17</v>
@@ -4801,7 +4798,7 @@
     </row>
     <row r="85" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>12</v>
@@ -4822,10 +4819,10 @@
         <v>0.13</v>
       </c>
       <c r="H85" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="I85" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="I85" s="15" t="s">
-        <v>326</v>
       </c>
       <c r="J85" s="11" t="s">
         <v>17</v>
@@ -4839,7 +4836,7 @@
     </row>
     <row r="86" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>12</v>
@@ -4863,7 +4860,7 @@
         <v>41</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J86" s="11" t="s">
         <v>17</v>
@@ -4877,7 +4874,7 @@
     </row>
     <row r="87" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>12</v>
@@ -4901,7 +4898,7 @@
         <v>41</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J87" s="11" t="s">
         <v>17</v>
@@ -4915,7 +4912,7 @@
     </row>
     <row r="88" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>40</v>
@@ -4936,16 +4933,16 @@
         <v>0.128</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I88" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="J88" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K88" s="11" t="s">
         <v>329</v>
-      </c>
-      <c r="J88" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K88" s="11" t="s">
-        <v>330</v>
       </c>
       <c r="L88" s="11" t="s">
         <v>18</v>
@@ -4953,7 +4950,7 @@
     </row>
     <row r="89" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>40</v>
@@ -4965,7 +4962,7 @@
         <v>67</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F89" s="1">
         <v>1</v>
@@ -4974,10 +4971,10 @@
         <v>0.125</v>
       </c>
       <c r="H89" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J89" s="11" t="s">
         <v>24</v>
@@ -4991,7 +4988,7 @@
     </row>
     <row r="90" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>12</v>
@@ -5015,7 +5012,7 @@
         <v>52</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>17</v>
@@ -5029,7 +5026,7 @@
     </row>
     <row r="91" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>12</v>
@@ -5050,10 +5047,10 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H91" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="I91" s="15" t="s">
         <v>333</v>
-      </c>
-      <c r="I91" s="15" t="s">
-        <v>334</v>
       </c>
       <c r="J91" s="11" t="s">
         <v>17</v>
@@ -5067,7 +5064,7 @@
     </row>
     <row r="92" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>12</v>
@@ -5088,13 +5085,13 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H92" s="11" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="I92" s="15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K92" s="11" t="s">
         <v>18</v>
@@ -5105,7 +5102,7 @@
     </row>
     <row r="93" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>12</v>
@@ -5126,13 +5123,13 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I93" s="15" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K93" s="11" t="s">
         <v>18</v>
@@ -5143,7 +5140,7 @@
     </row>
     <row r="94" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>12</v>
@@ -5155,7 +5152,7 @@
         <v>30</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F94" s="1">
         <v>1</v>
@@ -5164,16 +5161,16 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I94" s="15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K94" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L94" s="11" t="s">
         <v>82</v>
@@ -5181,7 +5178,7 @@
     </row>
     <row r="95" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>12</v>
@@ -5193,7 +5190,7 @@
         <v>222</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F95" s="1">
         <v>1</v>
@@ -5202,10 +5199,10 @@
         <v>0.13</v>
       </c>
       <c r="H95" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="I95" s="15" t="s">
         <v>338</v>
-      </c>
-      <c r="I95" s="15" t="s">
-        <v>339</v>
       </c>
       <c r="J95" s="11" t="s">
         <v>17</v>
@@ -5219,7 +5216,7 @@
     </row>
     <row r="96" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>12</v>
@@ -5228,7 +5225,7 @@
         <v>89.088999999999999</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E96" s="10" t="s">
         <v>116</v>
@@ -5240,10 +5237,10 @@
         <v>0.129</v>
       </c>
       <c r="H96" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="I96" s="15" t="s">
         <v>340</v>
-      </c>
-      <c r="I96" s="15" t="s">
-        <v>341</v>
       </c>
       <c r="J96" s="11" t="s">
         <v>17</v>
@@ -5257,7 +5254,7 @@
     </row>
     <row r="97" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>12</v>
@@ -5281,13 +5278,13 @@
         <v>32</v>
       </c>
       <c r="I97" s="15" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J97" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K97" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L97" s="11" t="s">
         <v>82</v>
@@ -5295,7 +5292,7 @@
     </row>
     <row r="98" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>12</v>
@@ -5316,13 +5313,13 @@
         <v>0.13800000000000001</v>
       </c>
       <c r="H98" s="11" t="s">
+        <v>342</v>
+      </c>
+      <c r="I98" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="I98" s="15" t="s">
-        <v>344</v>
-      </c>
       <c r="J98" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K98" s="11" t="s">
         <v>18</v>
@@ -5333,7 +5330,7 @@
     </row>
     <row r="99" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>12</v>
@@ -5345,7 +5342,7 @@
         <v>51</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F99" s="1">
         <v>1</v>
@@ -5354,10 +5351,10 @@
         <v>0.13</v>
       </c>
       <c r="H99" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="I99" s="15" t="s">
         <v>345</v>
-      </c>
-      <c r="I99" s="15" t="s">
-        <v>346</v>
       </c>
       <c r="J99" s="11" t="s">
         <v>18</v>
@@ -5371,7 +5368,7 @@
     </row>
     <row r="100" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>12</v>
@@ -5392,10 +5389,10 @@
         <v>0.125</v>
       </c>
       <c r="H100" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="I100" s="15" t="s">
         <v>347</v>
-      </c>
-      <c r="I100" s="15" t="s">
-        <v>348</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>18</v>
@@ -5409,7 +5406,7 @@
     </row>
     <row r="101" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>21</v>
@@ -5430,10 +5427,10 @@
         <v>0.12</v>
       </c>
       <c r="H101" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I101" s="15" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J101" s="11" t="s">
         <v>18</v>
@@ -5447,7 +5444,7 @@
     </row>
     <row r="102" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>21</v>
@@ -5459,7 +5456,7 @@
         <v>51</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F102" s="1">
         <v>1</v>
@@ -5468,10 +5465,10 @@
         <v>0.125</v>
       </c>
       <c r="H102" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="I102" s="15" t="s">
         <v>350</v>
-      </c>
-      <c r="I102" s="15" t="s">
-        <v>351</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>18</v>
@@ -5485,7 +5482,7 @@
     </row>
     <row r="103" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>12</v>
@@ -5497,7 +5494,7 @@
         <v>51</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F103" s="1">
         <v>1</v>
@@ -5506,10 +5503,10 @@
         <v>0.13</v>
       </c>
       <c r="H103" s="11" t="s">
+        <v>351</v>
+      </c>
+      <c r="I103" s="15" t="s">
         <v>352</v>
-      </c>
-      <c r="I103" s="15" t="s">
-        <v>353</v>
       </c>
       <c r="J103" s="11" t="s">
         <v>18</v>
@@ -5523,7 +5520,7 @@
     </row>
     <row r="104" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>12</v>
@@ -5535,7 +5532,7 @@
         <v>51</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F104" s="1">
         <v>1</v>
@@ -5544,10 +5541,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H104" s="11" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I104" s="15" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J104" s="11" t="s">
         <v>18</v>
@@ -5561,7 +5558,7 @@
     </row>
     <row r="105" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>12</v>
@@ -5582,10 +5579,10 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H105" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I105" s="15" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J105" s="11" t="s">
         <v>17</v>
@@ -5599,7 +5596,7 @@
     </row>
     <row r="106" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>12</v>
@@ -5620,10 +5617,10 @@
         <v>0.13</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I106" s="15" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>17</v>
@@ -5637,7 +5634,7 @@
     </row>
     <row r="107" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>12</v>
@@ -5658,16 +5655,16 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H107" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I107" s="15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J107" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K107" s="11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L107" s="11" t="s">
         <v>18</v>
@@ -5675,7 +5672,7 @@
     </row>
     <row r="108" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>12</v>
@@ -5687,7 +5684,7 @@
         <v>30</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F108" s="1">
         <v>1</v>
@@ -5696,10 +5693,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H108" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I108" s="15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J108" s="11" t="s">
         <v>17</v>
@@ -5713,7 +5710,7 @@
     </row>
     <row r="109" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>40</v>
@@ -5734,10 +5731,10 @@
         <v>0.125</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="I109" s="15" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J109" s="11" t="s">
         <v>26</v>
@@ -5751,7 +5748,7 @@
     </row>
     <row r="110" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>21</v>
@@ -5772,10 +5769,10 @@
         <v>0.12</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="I110" s="15" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>24</v>
@@ -5784,12 +5781,12 @@
         <v>43</v>
       </c>
       <c r="L110" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>40</v>
@@ -5801,7 +5798,7 @@
         <v>112</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F111" s="1">
         <v>1</v>
@@ -5813,7 +5810,7 @@
         <v>47</v>
       </c>
       <c r="I111" s="15" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J111" s="11" t="s">
         <v>24</v>
@@ -5827,7 +5824,7 @@
     </row>
     <row r="112" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>40</v>
@@ -5839,7 +5836,7 @@
         <v>51</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F112" s="1">
         <v>1</v>
@@ -5848,10 +5845,10 @@
         <v>0.12</v>
       </c>
       <c r="H112" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I112" s="15" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J112" s="11" t="s">
         <v>24</v>
@@ -5865,7 +5862,7 @@
     </row>
     <row r="113" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>12</v>
@@ -5886,10 +5883,10 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="H113" s="11" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I113" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J113" s="11" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Corrige categorias de 5 vinhos e troca a foto do Winemaker Secret Rosé
Categorias, conforme a planilha revisada: Fonte da Perdiz Branco D.O.C.
(Tinto -> Branco), Ique Vegano (Branco -> Tinto), Martha's Moscatel do Douro
(Tinto -> Sobremesa), Nobili D'Italia Montepulciano D'Abruzzo (Branco ->
Tinto) e Vezzani Montepulciano (Rosé -> Tinto). A aba Sobremesa passa a ter
2 vinhos.

A foto do Winemaker Secret Rosé estava errada; a nova foi enviada pelo dono
e salva no padrão do site (900x900, JPEG q82).

Continuam sem ser copiados da planilha os valores que parecem erro de
digitação: país "Aegentina" (Bodega Torrontés), Profugo Malbec como Branco
(é tinto, confirmado) e uva Cabernet Sauvignon no Isla Negra Carménère.
Cache do service worker v13 -> v14.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Produto_Todos_Vinhos.xlsx
+++ b/Planilha_Produto_Todos_Vinhos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f88f9e9a0b886b5b/Nova_Vinho_Harmonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F02A2EAB-7882-4827-A1EA-6D7C8C307BE7}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A816421A-9114-492D-8730-FC465510F5F4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2858,7 +2858,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="84" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:12" ht="67.2" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>136</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>146</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C38" s="7">
         <v>50.787299999999995</v>
@@ -3276,12 +3276,12 @@
         <v>169</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>170</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C45" s="7">
         <v>50.982399999999998</v>
@@ -3580,7 +3580,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>200</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>205</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>12</v>
+        <v>194</v>
       </c>
       <c r="C55" s="7">
         <v>70.801599999999993</v>
@@ -4345,7 +4345,7 @@
         <v>226</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C73" s="7">
         <v>67.62</v>
@@ -5409,7 +5409,7 @@
         <v>262</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C101" s="7">
         <v>91.322000000000003</v>

</xml_diff>

<commit_message>
Adiciona dois vinhos novos: Paso de Los Andes Carmenere Preto e Sangiovese Toscana
Cadastrados na planilha pelo dono, com fotos enviadas por ele (900x900,
JPEG q82): Paso de Los Andes Carmenere Preto (Chile, R$ 58,87, 13%) e
Sangiovese Toscana Rifugio del Vescovo (Italia, R$ 95,65, 12,5%), ambos com
estoque inicial 4 e inseridos em ordem alfabetica. O nome do Sangiovese vem
sem espaco na planilha ("SangioveseToscana"); no site vai com espaco.

A harmonizacao Funghi (nova) ganha o icone de cogumelo, em vez do icone
padrao de taca. Planilha atualizada junto. Catalogo: 112 -> 114 vinhos. Cache
do service worker v15 -> v16.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Produto_Todos_Vinhos.xlsx
+++ b/Planilha_Produto_Todos_Vinhos.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f88f9e9a0b886b5b/Nova_Vinho_Harmonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A816421A-9114-492D-8730-FC465510F5F4}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CB698A5-8955-4034-92F5-3A510F773AD7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="374">
   <si>
     <t>Nome Vinho</t>
   </si>
@@ -1193,6 +1206,27 @@
   <si>
     <t>Secreta</t>
   </si>
+  <si>
+    <t xml:space="preserve">Massas </t>
+  </si>
+  <si>
+    <t>Paso de Los Andes Carménère Preto</t>
+  </si>
+  <si>
+    <t>Vale do Curicó</t>
+  </si>
+  <si>
+    <t>SangioveseToscana Rifugio del Vescovo</t>
+  </si>
+  <si>
+    <t>O Rifugio del Vescovo Sangiovese Toscana traz um pouco do charme e da tradição italiana para a sua mesa. É aquele vinho que convida a desacelerar, reunir os amigos e transformar um jantar simples em um momento especial.</t>
+  </si>
+  <si>
+    <t>O Paso de Los Andes Carménère é aquele vinho chileno que combina com momentos descontraídos e boas conversas à mesa. Com seu estilo macio, agradável e versátil, é uma ótima escolha para transformar refeições do dia a dia em experiências especiais.</t>
+  </si>
+  <si>
+    <t>Funghi</t>
+  </si>
 </sst>
 </file>
 
@@ -1253,7 +1287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1332,11 +1366,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1373,6 +1444,15 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1589,7 +1669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.88671875" style="4" customWidth="1"/>
@@ -5861,41 +5941,117 @@
       </c>
     </row>
     <row r="113" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A113" s="2" t="s">
+      <c r="A113" s="24" t="s">
         <v>279</v>
       </c>
-      <c r="B113" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C113" s="7">
+      <c r="B113" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C113" s="25">
         <v>69.695999999999998</v>
       </c>
-      <c r="D113" s="2" t="s">
+      <c r="D113" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="E113" s="10" t="s">
+      <c r="E113" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="F113" s="1">
-        <v>1</v>
-      </c>
-      <c r="G113" s="22">
+      <c r="F113" s="27">
+        <v>1</v>
+      </c>
+      <c r="G113" s="28">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="H113" s="11" t="s">
+      <c r="H113" s="29" t="s">
         <v>337</v>
       </c>
-      <c r="I113" s="15" t="s">
+      <c r="I113" s="30" t="s">
         <v>362</v>
       </c>
-      <c r="J113" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K113" s="11" t="s">
+      <c r="J113" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="K113" s="29" t="s">
         <v>173</v>
       </c>
-      <c r="L113" s="11" t="s">
+      <c r="L113" s="29" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C114" s="5">
+        <v>95.65</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F114" s="1">
+        <v>4</v>
+      </c>
+      <c r="G114" s="17">
+        <v>0.125</v>
+      </c>
+      <c r="H114" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="I114" s="14" t="s">
+        <v>371</v>
+      </c>
+      <c r="J114" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="K114" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="L114" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C115" s="5">
+        <v>58.87</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F115" s="1">
+        <v>4</v>
+      </c>
+      <c r="G115" s="19">
+        <v>0.13</v>
+      </c>
+      <c r="H115" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="I115" s="14" t="s">
+        <v>372</v>
+      </c>
+      <c r="J115" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="K115" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="L115" s="12" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige o nome do Paso de Los Andes Cabernet Sauvignon e o pais do Baron Philippe
Acertos feitos na planilha:
- "Pao de Los Andes Cabernet Sauvignon" passa a "Paso de Los Andes Cabernet
  Sauvignon". O comeco da descricao repetia o mesmo erro (a planilha ainda tem
  "Pao" nesse texto) e tambem foi corrigido. O slug e o arquivo da foto NAO
  mudam de proposito: o estoque no banco, os pedidos ja gravados e os carrinhos
  guardados nos celulares usam o slug; mudar criaria uma linha de estoque nova.
- Baron Philippe de Rothschild Reserva Especial Merlot: pais Franca -> Chile
  (a regiao na planilha e Vale Central). Franca 13 -> 12 vinhos e Chile
  16 -> 17 nos filtros.

Planilha atualizada junto. Cache do service worker v18 -> v19.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Produto_Todos_Vinhos.xlsx
+++ b/Planilha_Produto_Todos_Vinhos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f88f9e9a0b886b5b/Nova_Vinho_Harmonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CB698A5-8955-4034-92F5-3A510F773AD7}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB928953-70EC-4967-8D69-274458626F46}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="375">
   <si>
     <t>Nome Vinho</t>
   </si>
@@ -802,9 +802,6 @@
     <t>Paso de Los Andes Reserva Tinto</t>
   </si>
   <si>
-    <t>Pao de Los Andes Cabernet Sauvignon</t>
-  </si>
-  <si>
     <t>Passo de Los Andes Carménère</t>
   </si>
   <si>
@@ -1226,6 +1223,12 @@
   </si>
   <si>
     <t>Funghi</t>
+  </si>
+  <si>
+    <t>Paso de Los Andes Cabernet Sauvignon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chile </t>
   </si>
 </sst>
 </file>
@@ -1701,7 +1704,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -1961,7 +1964,7 @@
         <v>65.55</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>45</v>
+        <v>374</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>46</v>
@@ -2216,7 +2219,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>75</v>
       </c>
@@ -3014,7 +3017,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>140</v>
       </c>
@@ -3698,7 +3701,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>202</v>
       </c>
@@ -3762,13 +3765,13 @@
         <v>15</v>
       </c>
       <c r="I55" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="J55" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="J55" s="11" t="s">
+      <c r="K55" s="11" t="s">
         <v>281</v>
-      </c>
-      <c r="K55" s="11" t="s">
-        <v>282</v>
       </c>
       <c r="L55" s="11" t="s">
         <v>199</v>
@@ -3800,7 +3803,7 @@
         <v>32</v>
       </c>
       <c r="I56" s="15" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J56" s="11" t="s">
         <v>17</v>
@@ -3835,10 +3838,10 @@
         <v>0.115</v>
       </c>
       <c r="H57" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="I57" s="15" t="s">
         <v>284</v>
-      </c>
-      <c r="I57" s="15" t="s">
-        <v>285</v>
       </c>
       <c r="J57" s="11" t="s">
         <v>24</v>
@@ -3873,10 +3876,10 @@
         <v>0.14499999999999999</v>
       </c>
       <c r="H58" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="I58" s="15" t="s">
         <v>286</v>
-      </c>
-      <c r="I58" s="15" t="s">
-        <v>287</v>
       </c>
       <c r="J58" s="11" t="s">
         <v>17</v>
@@ -3911,10 +3914,10 @@
         <v>0.13</v>
       </c>
       <c r="H59" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="I59" s="15" t="s">
         <v>288</v>
-      </c>
-      <c r="I59" s="15" t="s">
-        <v>289</v>
       </c>
       <c r="J59" s="11" t="s">
         <v>17</v>
@@ -3949,10 +3952,10 @@
         <v>0.125</v>
       </c>
       <c r="H60" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="I60" s="15" t="s">
         <v>290</v>
-      </c>
-      <c r="I60" s="15" t="s">
-        <v>291</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>24</v>
@@ -3961,7 +3964,7 @@
         <v>43</v>
       </c>
       <c r="L60" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3990,7 +3993,7 @@
         <v>47</v>
       </c>
       <c r="I61" s="15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J61" s="11" t="s">
         <v>17</v>
@@ -4028,7 +4031,7 @@
         <v>47</v>
       </c>
       <c r="I62" s="15" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J62" s="11" t="s">
         <v>26</v>
@@ -4066,7 +4069,7 @@
         <v>47</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>17</v>
@@ -4104,13 +4107,13 @@
         <v>32</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J64" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K64" s="11" t="s">
         <v>281</v>
-      </c>
-      <c r="K64" s="11" t="s">
-        <v>282</v>
       </c>
       <c r="L64" s="11" t="s">
         <v>199</v>
@@ -4139,13 +4142,13 @@
         <v>0.13</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I65" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="J65" s="11" t="s">
         <v>297</v>
-      </c>
-      <c r="J65" s="11" t="s">
-        <v>298</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>18</v>
@@ -4177,10 +4180,10 @@
         <v>0.13</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I66" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J66" s="11" t="s">
         <v>17</v>
@@ -4215,10 +4218,10 @@
         <v>0.13</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I67" s="15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J67" s="11" t="s">
         <v>17</v>
@@ -4253,16 +4256,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H68" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="I68" s="15" t="s">
         <v>301</v>
       </c>
-      <c r="I68" s="15" t="s">
+      <c r="J68" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K68" s="11" t="s">
         <v>302</v>
-      </c>
-      <c r="J68" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K68" s="11" t="s">
-        <v>303</v>
       </c>
       <c r="L68" s="11" t="s">
         <v>82</v>
@@ -4291,10 +4294,10 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H69" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="I69" s="15" t="s">
         <v>304</v>
-      </c>
-      <c r="I69" s="15" t="s">
-        <v>305</v>
       </c>
       <c r="J69" s="11" t="s">
         <v>17</v>
@@ -4329,10 +4332,10 @@
         <v>0.13</v>
       </c>
       <c r="H70" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="I70" s="15" t="s">
         <v>306</v>
-      </c>
-      <c r="I70" s="15" t="s">
-        <v>307</v>
       </c>
       <c r="J70" s="11" t="s">
         <v>17</v>
@@ -4367,10 +4370,10 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H71" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J71" s="11" t="s">
         <v>17</v>
@@ -4408,7 +4411,7 @@
         <v>41</v>
       </c>
       <c r="I72" s="15" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>17</v>
@@ -4443,10 +4446,10 @@
         <v>0.13</v>
       </c>
       <c r="H73" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="I73" s="15" t="s">
         <v>310</v>
-      </c>
-      <c r="I73" s="15" t="s">
-        <v>311</v>
       </c>
       <c r="J73" s="11" t="s">
         <v>18</v>
@@ -4481,10 +4484,10 @@
         <v>0.11</v>
       </c>
       <c r="H74" s="11" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I74" s="15" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="J74" s="11" t="s">
         <v>24</v>
@@ -4522,10 +4525,10 @@
         <v>47</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K75" s="11" t="s">
         <v>18</v>
@@ -4560,7 +4563,7 @@
         <v>47</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>17</v>
@@ -4574,7 +4577,7 @@
     </row>
     <row r="77" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>232</v>
+        <v>373</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>12</v>
@@ -4598,7 +4601,7 @@
         <v>47</v>
       </c>
       <c r="I77" s="15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J77" s="11" t="s">
         <v>17</v>
@@ -4612,7 +4615,7 @@
     </row>
     <row r="78" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>12</v>
@@ -4636,7 +4639,7 @@
         <v>47</v>
       </c>
       <c r="I78" s="15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J78" s="11" t="s">
         <v>17</v>
@@ -4650,7 +4653,7 @@
     </row>
     <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>12</v>
@@ -4671,10 +4674,10 @@
         <v>0.127</v>
       </c>
       <c r="H79" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="I79" s="15" t="s">
         <v>317</v>
-      </c>
-      <c r="I79" s="15" t="s">
-        <v>318</v>
       </c>
       <c r="J79" s="11" t="s">
         <v>17</v>
@@ -4688,7 +4691,7 @@
     </row>
     <row r="80" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>12</v>
@@ -4700,7 +4703,7 @@
         <v>30</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F80" s="1">
         <v>1</v>
@@ -4709,16 +4712,16 @@
         <v>0.125</v>
       </c>
       <c r="H80" s="11" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I80" s="15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J80" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K80" s="11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="L80" s="11" t="s">
         <v>82</v>
@@ -4726,7 +4729,7 @@
     </row>
     <row r="81" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>12</v>
@@ -4750,13 +4753,13 @@
         <v>47</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J81" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K81" s="11" t="s">
         <v>281</v>
-      </c>
-      <c r="K81" s="11" t="s">
-        <v>282</v>
       </c>
       <c r="L81" s="11" t="s">
         <v>199</v>
@@ -4764,7 +4767,7 @@
     </row>
     <row r="82" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>40</v>
@@ -4785,10 +4788,10 @@
         <v>0.12</v>
       </c>
       <c r="H82" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J82" s="11" t="s">
         <v>26</v>
@@ -4802,7 +4805,7 @@
     </row>
     <row r="83" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>119</v>
@@ -4826,7 +4829,7 @@
         <v>22</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J83" s="11" t="s">
         <v>26</v>
@@ -4840,7 +4843,7 @@
     </row>
     <row r="84" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>119</v>
@@ -4864,7 +4867,7 @@
         <v>22</v>
       </c>
       <c r="I84" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J84" s="11" t="s">
         <v>17</v>
@@ -4878,7 +4881,7 @@
     </row>
     <row r="85" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>12</v>
@@ -4899,10 +4902,10 @@
         <v>0.13</v>
       </c>
       <c r="H85" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="I85" s="15" t="s">
         <v>324</v>
-      </c>
-      <c r="I85" s="15" t="s">
-        <v>325</v>
       </c>
       <c r="J85" s="11" t="s">
         <v>17</v>
@@ -4916,7 +4919,7 @@
     </row>
     <row r="86" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>12</v>
@@ -4940,7 +4943,7 @@
         <v>41</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="J86" s="11" t="s">
         <v>17</v>
@@ -4954,7 +4957,7 @@
     </row>
     <row r="87" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>12</v>
@@ -4978,7 +4981,7 @@
         <v>41</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J87" s="11" t="s">
         <v>17</v>
@@ -4992,7 +4995,7 @@
     </row>
     <row r="88" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>40</v>
@@ -5013,16 +5016,16 @@
         <v>0.128</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I88" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="J88" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K88" s="11" t="s">
         <v>328</v>
-      </c>
-      <c r="J88" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K88" s="11" t="s">
-        <v>329</v>
       </c>
       <c r="L88" s="11" t="s">
         <v>18</v>
@@ -5030,7 +5033,7 @@
     </row>
     <row r="89" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>40</v>
@@ -5042,7 +5045,7 @@
         <v>67</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F89" s="1">
         <v>1</v>
@@ -5051,10 +5054,10 @@
         <v>0.125</v>
       </c>
       <c r="H89" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J89" s="11" t="s">
         <v>24</v>
@@ -5068,7 +5071,7 @@
     </row>
     <row r="90" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>12</v>
@@ -5092,7 +5095,7 @@
         <v>52</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>17</v>
@@ -5106,7 +5109,7 @@
     </row>
     <row r="91" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>12</v>
@@ -5127,10 +5130,10 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H91" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="I91" s="15" t="s">
         <v>332</v>
-      </c>
-      <c r="I91" s="15" t="s">
-        <v>333</v>
       </c>
       <c r="J91" s="11" t="s">
         <v>17</v>
@@ -5144,7 +5147,7 @@
     </row>
     <row r="92" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>12</v>
@@ -5165,13 +5168,13 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H92" s="11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="I92" s="15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K92" s="11" t="s">
         <v>18</v>
@@ -5182,7 +5185,7 @@
     </row>
     <row r="93" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>12</v>
@@ -5203,13 +5206,13 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I93" s="15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K93" s="11" t="s">
         <v>18</v>
@@ -5220,7 +5223,7 @@
     </row>
     <row r="94" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>12</v>
@@ -5232,7 +5235,7 @@
         <v>30</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F94" s="1">
         <v>1</v>
@@ -5241,16 +5244,16 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I94" s="15" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K94" s="11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="L94" s="11" t="s">
         <v>82</v>
@@ -5258,7 +5261,7 @@
     </row>
     <row r="95" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>12</v>
@@ -5270,7 +5273,7 @@
         <v>222</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F95" s="1">
         <v>1</v>
@@ -5279,10 +5282,10 @@
         <v>0.13</v>
       </c>
       <c r="H95" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="I95" s="15" t="s">
         <v>337</v>
-      </c>
-      <c r="I95" s="15" t="s">
-        <v>338</v>
       </c>
       <c r="J95" s="11" t="s">
         <v>17</v>
@@ -5296,7 +5299,7 @@
     </row>
     <row r="96" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>12</v>
@@ -5305,7 +5308,7 @@
         <v>89.088999999999999</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E96" s="10" t="s">
         <v>116</v>
@@ -5317,10 +5320,10 @@
         <v>0.129</v>
       </c>
       <c r="H96" s="11" t="s">
+        <v>338</v>
+      </c>
+      <c r="I96" s="15" t="s">
         <v>339</v>
-      </c>
-      <c r="I96" s="15" t="s">
-        <v>340</v>
       </c>
       <c r="J96" s="11" t="s">
         <v>17</v>
@@ -5334,7 +5337,7 @@
     </row>
     <row r="97" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>12</v>
@@ -5346,7 +5349,7 @@
         <v>30</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F97" s="1">
         <v>1</v>
@@ -5358,13 +5361,13 @@
         <v>32</v>
       </c>
       <c r="I97" s="15" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J97" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K97" s="11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="L97" s="11" t="s">
         <v>82</v>
@@ -5372,7 +5375,7 @@
     </row>
     <row r="98" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>12</v>
@@ -5393,13 +5396,13 @@
         <v>0.13800000000000001</v>
       </c>
       <c r="H98" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="I98" s="15" t="s">
         <v>342</v>
       </c>
-      <c r="I98" s="15" t="s">
-        <v>343</v>
-      </c>
       <c r="J98" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K98" s="11" t="s">
         <v>18</v>
@@ -5410,7 +5413,7 @@
     </row>
     <row r="99" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>12</v>
@@ -5422,7 +5425,7 @@
         <v>51</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F99" s="1">
         <v>1</v>
@@ -5431,10 +5434,10 @@
         <v>0.13</v>
       </c>
       <c r="H99" s="11" t="s">
+        <v>343</v>
+      </c>
+      <c r="I99" s="15" t="s">
         <v>344</v>
-      </c>
-      <c r="I99" s="15" t="s">
-        <v>345</v>
       </c>
       <c r="J99" s="11" t="s">
         <v>18</v>
@@ -5448,7 +5451,7 @@
     </row>
     <row r="100" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>12</v>
@@ -5469,10 +5472,10 @@
         <v>0.125</v>
       </c>
       <c r="H100" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="I100" s="15" t="s">
         <v>346</v>
-      </c>
-      <c r="I100" s="15" t="s">
-        <v>347</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>18</v>
@@ -5486,7 +5489,7 @@
     </row>
     <row r="101" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>12</v>
@@ -5507,10 +5510,10 @@
         <v>0.12</v>
       </c>
       <c r="H101" s="12" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I101" s="15" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J101" s="11" t="s">
         <v>18</v>
@@ -5524,7 +5527,7 @@
     </row>
     <row r="102" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>21</v>
@@ -5536,7 +5539,7 @@
         <v>51</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F102" s="1">
         <v>1</v>
@@ -5545,10 +5548,10 @@
         <v>0.125</v>
       </c>
       <c r="H102" s="11" t="s">
+        <v>348</v>
+      </c>
+      <c r="I102" s="15" t="s">
         <v>349</v>
-      </c>
-      <c r="I102" s="15" t="s">
-        <v>350</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>18</v>
@@ -5562,7 +5565,7 @@
     </row>
     <row r="103" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>12</v>
@@ -5574,7 +5577,7 @@
         <v>51</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F103" s="1">
         <v>1</v>
@@ -5583,10 +5586,10 @@
         <v>0.13</v>
       </c>
       <c r="H103" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="I103" s="15" t="s">
         <v>351</v>
-      </c>
-      <c r="I103" s="15" t="s">
-        <v>352</v>
       </c>
       <c r="J103" s="11" t="s">
         <v>18</v>
@@ -5600,7 +5603,7 @@
     </row>
     <row r="104" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>12</v>
@@ -5612,7 +5615,7 @@
         <v>51</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F104" s="1">
         <v>1</v>
@@ -5621,10 +5624,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H104" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I104" s="15" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="J104" s="11" t="s">
         <v>18</v>
@@ -5638,7 +5641,7 @@
     </row>
     <row r="105" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>12</v>
@@ -5659,10 +5662,10 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H105" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I105" s="15" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J105" s="11" t="s">
         <v>17</v>
@@ -5676,7 +5679,7 @@
     </row>
     <row r="106" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>12</v>
@@ -5697,10 +5700,10 @@
         <v>0.13</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I106" s="15" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>17</v>
@@ -5714,7 +5717,7 @@
     </row>
     <row r="107" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>12</v>
@@ -5735,16 +5738,16 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H107" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I107" s="15" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J107" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K107" s="11" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L107" s="11" t="s">
         <v>18</v>
@@ -5752,7 +5755,7 @@
     </row>
     <row r="108" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>12</v>
@@ -5764,7 +5767,7 @@
         <v>30</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F108" s="1">
         <v>1</v>
@@ -5773,10 +5776,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H108" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I108" s="15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J108" s="11" t="s">
         <v>17</v>
@@ -5790,7 +5793,7 @@
     </row>
     <row r="109" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>40</v>
@@ -5811,10 +5814,10 @@
         <v>0.125</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I109" s="15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J109" s="11" t="s">
         <v>26</v>
@@ -5828,7 +5831,7 @@
     </row>
     <row r="110" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>21</v>
@@ -5849,10 +5852,10 @@
         <v>0.12</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I110" s="15" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>24</v>
@@ -5861,12 +5864,12 @@
         <v>43</v>
       </c>
       <c r="L110" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>40</v>
@@ -5878,7 +5881,7 @@
         <v>112</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F111" s="1">
         <v>1</v>
@@ -5890,7 +5893,7 @@
         <v>47</v>
       </c>
       <c r="I111" s="15" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J111" s="11" t="s">
         <v>24</v>
@@ -5904,7 +5907,7 @@
     </row>
     <row r="112" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>40</v>
@@ -5916,7 +5919,7 @@
         <v>51</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F112" s="1">
         <v>1</v>
@@ -5925,10 +5928,10 @@
         <v>0.12</v>
       </c>
       <c r="H112" s="12" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I112" s="15" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J112" s="11" t="s">
         <v>24</v>
@@ -5942,7 +5945,7 @@
     </row>
     <row r="113" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A113" s="24" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B113" s="24" t="s">
         <v>12</v>
@@ -5963,10 +5966,10 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="H113" s="29" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I113" s="30" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J113" s="29" t="s">
         <v>17</v>
@@ -5980,7 +5983,7 @@
     </row>
     <row r="114" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>12</v>
@@ -6004,10 +6007,10 @@
         <v>52</v>
       </c>
       <c r="I114" s="14" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="J114" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="K114" s="12" t="s">
         <v>155</v>
@@ -6018,7 +6021,7 @@
     </row>
     <row r="115" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>12</v>
@@ -6039,16 +6042,16 @@
         <v>0.13</v>
       </c>
       <c r="H115" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I115" s="14" t="s">
+        <v>371</v>
+      </c>
+      <c r="J115" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="K115" s="12" t="s">
         <v>372</v>
-      </c>
-      <c r="J115" s="12" t="s">
-        <v>303</v>
-      </c>
-      <c r="K115" s="12" t="s">
-        <v>373</v>
       </c>
       <c r="L115" s="12" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Adiciona dois vinhos: Chateau Le Dragon e Da Pipa Frisante Rose
Cadastrados na planilha pelo dono, com fotos enviadas por ele (900x900, JPEG
q82), textos e dados lidos direto da planilha: Chateau Le Dragon (Tinto,
Franca, R$ 64,82, 13%, Cordeiro/Carnes/Queijos) e Da Pipa Frisante Rose (Rose,
Portugal, R$ 42,78, 11,5%, Saladas/Peixes/Frutos do Mar), ambos com estoque
inicial 4 e em ordem alfabetica. O Da Pipa ja existiu na loja e tinha sido
retirado; volta com preco e foto novos. Nenhuma linha de estoque antiga existia
para esse codigo (a regra de estoque foi criada depois da retirada), entao o
estoque comeca em 4.

Catalogo: 114 -> 116 vinhos. Cache do service worker v20 -> v21.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Produto_Todos_Vinhos.xlsx
+++ b/Planilha_Produto_Todos_Vinhos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f88f9e9a0b886b5b/Nova_Vinho_Harmonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB928953-70EC-4967-8D69-274458626F46}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{5D3ADACB-3E5F-4985-B9C2-EFA16530B4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2A808DB-F4DF-4186-BDFA-0F8F1534C658}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="377">
   <si>
     <t>Nome Vinho</t>
   </si>
@@ -209,9 +209,6 @@
     <t>Bodega Torrontés</t>
   </si>
   <si>
-    <t>Aegentina</t>
-  </si>
-  <si>
     <t>Torrontés</t>
   </si>
   <si>
@@ -225,9 +222,6 @@
   </si>
   <si>
     <t>Bridão Merlot</t>
-  </si>
-  <si>
-    <t>Imperial</t>
   </si>
   <si>
     <t>O Bridão Merlot 2017 é um tinto de perfil redondo e convidativo, com a Merlot mostrando seu lado mais macio: frutas vermelhas e negras maduras, leve toque de especiarias e uma textura aveludada que deixa o vinho fácil de beber.</t>
@@ -1229,6 +1223,18 @@
   </si>
   <si>
     <t xml:space="preserve">Chile </t>
+  </si>
+  <si>
+    <t>Château Le Dragon</t>
+  </si>
+  <si>
+    <t>Da Pipa Frisante Rosé</t>
+  </si>
+  <si>
+    <t>O Château Le Dragon traz a tradição e a elegância dos vinhos franceses para momentos especiais. É uma excelente companhia para jantares a dois, almoços em família e encontros com amigos, harmonizando com carnes assadas, massas ao molho encorpado, risotos de cogumelos e queijos maturados. Um vinho para apreciar sem pressa, transformar uma refeição em uma experiência e celebrar o prazer de estar à mesa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O Da Pipa Frisante Rosé é aquele vinho que combina com dias ensolarados, encontros descontraídos e momentos que merecem um toque de alegria. Com sua leveza, frescor e delicadas borbulhas, é perfeito para um happy hour, um almoço ao ar livre, um fim de tarde na varanda ou uma reunião com amigos. </t>
   </si>
 </sst>
 </file>
@@ -1672,7 +1678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.88671875" style="4" customWidth="1"/>
@@ -1704,7 +1710,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -1964,7 +1970,7 @@
         <v>65.55</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>46</v>
@@ -2078,10 +2084,10 @@
         <v>56.883499999999998</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>59</v>
       </c>
       <c r="F11" s="1">
         <v>1</v>
@@ -2090,10 +2096,10 @@
         <v>0.128</v>
       </c>
       <c r="H11" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" s="14" t="s">
         <v>60</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>61</v>
       </c>
       <c r="J11" s="12" t="s">
         <v>54</v>
@@ -2102,12 +2108,12 @@
         <v>43</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
@@ -2116,7 +2122,7 @@
         <v>103.5585</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>46</v>
@@ -2131,7 +2137,7 @@
         <v>22</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J12" s="12" t="s">
         <v>17</v>
@@ -2145,7 +2151,7 @@
     </row>
     <row r="13" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>12</v>
@@ -2154,10 +2160,10 @@
         <v>75.302400000000006</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F13" s="1">
         <v>1</v>
@@ -2166,10 +2172,10 @@
         <v>0.13300000000000001</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J13" s="12" t="s">
         <v>17</v>
@@ -2183,7 +2189,7 @@
     </row>
     <row r="14" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
@@ -2195,7 +2201,7 @@
         <v>51</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F14" s="1">
         <v>1</v>
@@ -2204,10 +2210,10 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J14" s="12" t="s">
         <v>18</v>
@@ -2221,7 +2227,7 @@
     </row>
     <row r="15" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>12</v>
@@ -2233,7 +2239,7 @@
         <v>51</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
@@ -2242,16 +2248,16 @@
         <v>0.13</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J15" s="12" t="s">
         <v>26</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L15" s="12" t="s">
         <v>17</v>
@@ -2259,7 +2265,7 @@
     </row>
     <row r="16" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>12</v>
@@ -2280,13 +2286,13 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H16" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="12" t="s">
         <v>80</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>82</v>
       </c>
       <c r="K16" s="12" t="s">
         <v>17</v>
@@ -2297,7 +2303,7 @@
     </row>
     <row r="17" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>12</v>
@@ -2309,7 +2315,7 @@
         <v>30</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
@@ -2321,21 +2327,21 @@
         <v>37</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J17" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>40</v>
@@ -2347,7 +2353,7 @@
         <v>30</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
@@ -2359,7 +2365,7 @@
         <v>37</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J18" s="12" t="s">
         <v>54</v>
@@ -2373,7 +2379,7 @@
     </row>
     <row r="19" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>12</v>
@@ -2382,10 +2388,10 @@
         <v>47.701199999999993</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F19" s="1">
         <v>1</v>
@@ -2394,10 +2400,10 @@
         <v>0.125</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J19" s="12" t="s">
         <v>17</v>
@@ -2411,7 +2417,7 @@
     </row>
     <row r="20" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>40</v>
@@ -2423,7 +2429,7 @@
         <v>30</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F20" s="1">
         <v>1</v>
@@ -2435,7 +2441,7 @@
         <v>32</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J20" s="12" t="s">
         <v>24</v>
@@ -2449,7 +2455,7 @@
     </row>
     <row r="21" spans="1:12" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>12</v>
@@ -2470,10 +2476,10 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="J21" s="12" t="s">
         <v>49</v>
@@ -2487,7 +2493,7 @@
     </row>
     <row r="22" spans="1:12" ht="90" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>12</v>
@@ -2508,16 +2514,16 @@
         <v>0.13</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I22" s="20" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L22" s="12" t="s">
         <v>34</v>
@@ -2525,7 +2531,7 @@
     </row>
     <row r="23" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>12</v>
@@ -2546,16 +2552,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J23" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L23" s="12" t="s">
         <v>34</v>
@@ -2563,7 +2569,7 @@
     </row>
     <row r="24" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>12</v>
@@ -2572,10 +2578,10 @@
         <v>113.8626</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F24" s="1">
         <v>1</v>
@@ -2584,16 +2590,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L24" s="12" t="s">
         <v>34</v>
@@ -2601,7 +2607,7 @@
     </row>
     <row r="25" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>12</v>
@@ -2613,7 +2619,7 @@
         <v>51</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F25" s="1">
         <v>1</v>
@@ -2625,7 +2631,7 @@
         <v>52</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J25" s="12" t="s">
         <v>18</v>
@@ -2639,7 +2645,7 @@
     </row>
     <row r="26" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>12</v>
@@ -2663,7 +2669,7 @@
         <v>41</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>19</v>
@@ -2677,7 +2683,7 @@
     </row>
     <row r="27" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>12</v>
@@ -2686,10 +2692,10 @@
         <v>53.055999999999997</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F27" s="1">
         <v>1</v>
@@ -2701,13 +2707,13 @@
         <v>47</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J27" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L27" s="12" t="s">
         <v>34</v>
@@ -2715,7 +2721,7 @@
     </row>
     <row r="28" spans="1:12" ht="69.150000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>12</v>
@@ -2724,10 +2730,10 @@
         <v>58.928999999999995</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F28" s="1">
         <v>1</v>
@@ -2739,13 +2745,13 @@
         <v>47</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J28" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L28" s="12" t="s">
         <v>49</v>
@@ -2753,10 +2759,10 @@
     </row>
     <row r="29" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C29" s="7">
         <v>63.164999999999999</v>
@@ -2774,10 +2780,10 @@
         <v>0.115</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J29" s="12" t="s">
         <v>24</v>
@@ -2791,7 +2797,7 @@
     </row>
     <row r="30" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>40</v>
@@ -2800,10 +2806,10 @@
         <v>83.346000000000004</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F30" s="1">
         <v>1</v>
@@ -2812,10 +2818,10 @@
         <v>0.105</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J30" s="12" t="s">
         <v>24</v>
@@ -2829,7 +2835,7 @@
     </row>
     <row r="31" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>21</v>
@@ -2850,10 +2856,10 @@
         <v>0.115</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J31" s="12" t="s">
         <v>24</v>
@@ -2867,7 +2873,7 @@
     </row>
     <row r="32" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>12</v>
@@ -2888,10 +2894,10 @@
         <v>0.127</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J32" s="12" t="s">
         <v>17</v>
@@ -2900,12 +2906,12 @@
         <v>34</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>12</v>
@@ -2917,7 +2923,7 @@
         <v>30</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F33" s="1">
         <v>1</v>
@@ -2926,10 +2932,10 @@
         <v>0.123</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J33" s="12" t="s">
         <v>17</v>
@@ -2938,12 +2944,12 @@
         <v>49</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="67.2" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>12</v>
@@ -2964,10 +2970,10 @@
         <v>0.08</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I34" s="21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J34" s="12" t="s">
         <v>17</v>
@@ -2976,12 +2982,12 @@
         <v>34</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>12</v>
@@ -2990,10 +2996,10 @@
         <v>83.551999999999992</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F35" s="1">
         <v>1</v>
@@ -3005,7 +3011,7 @@
         <v>47</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J35" s="12" t="s">
         <v>17</v>
@@ -3014,12 +3020,12 @@
         <v>49</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>12</v>
@@ -3028,10 +3034,10 @@
         <v>49.927500000000002</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
@@ -3040,10 +3046,10 @@
         <v>0.13</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>17</v>
@@ -3052,12 +3058,12 @@
         <v>34</v>
       </c>
       <c r="L36" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>12</v>
@@ -3078,10 +3084,10 @@
         <v>0.13</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I37" s="14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J37" s="12" t="s">
         <v>19</v>
@@ -3095,7 +3101,7 @@
     </row>
     <row r="38" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>40</v>
@@ -3119,7 +3125,7 @@
         <v>15</v>
       </c>
       <c r="I38" s="14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>26</v>
@@ -3133,7 +3139,7 @@
     </row>
     <row r="39" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>21</v>
@@ -3145,7 +3151,7 @@
         <v>30</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F39" s="1">
         <v>1</v>
@@ -3154,10 +3160,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J39" s="12" t="s">
         <v>26</v>
@@ -3171,7 +3177,7 @@
     </row>
     <row r="40" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>12</v>
@@ -3180,10 +3186,10 @@
         <v>48.585000000000001</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F40" s="1">
         <v>1</v>
@@ -3192,24 +3198,24 @@
         <v>0.125</v>
       </c>
       <c r="H40" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="J40" s="12" t="s">
         <v>153</v>
-      </c>
-      <c r="I40" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="J40" s="12" t="s">
-        <v>155</v>
       </c>
       <c r="K40" s="12" t="s">
         <v>18</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>12</v>
@@ -3221,7 +3227,7 @@
         <v>13</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F41" s="1">
         <v>1</v>
@@ -3230,10 +3236,10 @@
         <v>0.14499999999999999</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J41" s="12" t="s">
         <v>17</v>
@@ -3247,7 +3253,7 @@
     </row>
     <row r="42" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>12</v>
@@ -3268,10 +3274,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J42" s="12" t="s">
         <v>19</v>
@@ -3285,7 +3291,7 @@
     </row>
     <row r="43" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>12</v>
@@ -3297,7 +3303,7 @@
         <v>51</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F43" s="1">
         <v>1</v>
@@ -3306,10 +3312,10 @@
         <v>0.13</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J43" s="12" t="s">
         <v>18</v>
@@ -3318,12 +3324,12 @@
         <v>34</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>12</v>
@@ -3344,24 +3350,24 @@
         <v>0.13</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J44" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>12</v>
@@ -3370,10 +3376,10 @@
         <v>50.982399999999998</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F45" s="1">
         <v>1</v>
@@ -3382,16 +3388,16 @@
         <v>0.128</v>
       </c>
       <c r="H45" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J45" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="I45" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="J45" s="12" t="s">
-        <v>173</v>
-      </c>
       <c r="K45" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="L45" s="12" t="s">
         <v>49</v>
@@ -3399,7 +3405,7 @@
     </row>
     <row r="46" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>12</v>
@@ -3408,10 +3414,10 @@
         <v>40.79</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F46" s="1">
         <v>1</v>
@@ -3423,21 +3429,21 @@
         <v>47</v>
       </c>
       <c r="I46" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="J46" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="K46" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="J46" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="K46" s="12" t="s">
-        <v>177</v>
-      </c>
       <c r="L46" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>12</v>
@@ -3461,21 +3467,21 @@
         <v>41</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="J47" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K47" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="L47" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>12</v>
@@ -3496,16 +3502,16 @@
         <v>0.13</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J48" s="12" t="s">
         <v>17</v>
       </c>
       <c r="K48" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="L48" s="12" t="s">
         <v>34</v>
@@ -3513,7 +3519,7 @@
     </row>
     <row r="49" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>12</v>
@@ -3525,7 +3531,7 @@
         <v>45</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F49" s="1">
         <v>1</v>
@@ -3534,24 +3540,24 @@
         <v>0.13</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J49" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L49" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>40</v>
@@ -3563,7 +3569,7 @@
         <v>51</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F50" s="1">
         <v>1</v>
@@ -3572,10 +3578,10 @@
         <v>0.08</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J50" s="12" t="s">
         <v>24</v>
@@ -3589,7 +3595,7 @@
     </row>
     <row r="51" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>12</v>
@@ -3601,7 +3607,7 @@
         <v>51</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F51" s="1">
         <v>1</v>
@@ -3610,16 +3616,16 @@
         <v>0.08</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J51" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K51" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="L51" s="12" t="s">
         <v>25</v>
@@ -3627,10 +3633,10 @@
     </row>
     <row r="52" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C52" s="7">
         <v>62.1</v>
@@ -3648,24 +3654,24 @@
         <v>0.155</v>
       </c>
       <c r="H52" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="I52" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="J52" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="I52" s="14" t="s">
+      <c r="K52" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="J52" s="12" t="s">
+      <c r="L52" s="12" t="s">
         <v>197</v>
-      </c>
-      <c r="K52" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="L52" s="12" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>12</v>
@@ -3674,10 +3680,10 @@
         <v>51.366</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F53" s="1">
         <v>1</v>
@@ -3686,13 +3692,13 @@
         <v>0.13</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K53" s="12" t="s">
         <v>17</v>
@@ -3703,7 +3709,7 @@
     </row>
     <row r="54" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>12</v>
@@ -3715,7 +3721,7 @@
         <v>30</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F54" s="1">
         <v>1</v>
@@ -3727,7 +3733,7 @@
         <v>32</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J54" s="12" t="s">
         <v>17</v>
@@ -3736,15 +3742,15 @@
         <v>34</v>
       </c>
       <c r="L54" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C55" s="7">
         <v>70.801599999999993</v>
@@ -3753,7 +3759,7 @@
         <v>13</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F55" s="1">
         <v>1</v>
@@ -3765,21 +3771,21 @@
         <v>15</v>
       </c>
       <c r="I55" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="J55" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="K55" s="11" t="s">
         <v>279</v>
       </c>
-      <c r="J55" s="11" t="s">
-        <v>280</v>
-      </c>
-      <c r="K55" s="11" t="s">
-        <v>281</v>
-      </c>
       <c r="L55" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="56" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>12</v>
@@ -3803,7 +3809,7 @@
         <v>32</v>
       </c>
       <c r="I56" s="15" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J56" s="11" t="s">
         <v>17</v>
@@ -3817,7 +3823,7 @@
     </row>
     <row r="57" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>40</v>
@@ -3829,7 +3835,7 @@
         <v>30</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F57" s="1">
         <v>1</v>
@@ -3838,10 +3844,10 @@
         <v>0.115</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I57" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="J57" s="11" t="s">
         <v>24</v>
@@ -3855,7 +3861,7 @@
     </row>
     <row r="58" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>12</v>
@@ -3867,7 +3873,7 @@
         <v>30</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F58" s="1">
         <v>1</v>
@@ -3876,10 +3882,10 @@
         <v>0.14499999999999999</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I58" s="15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J58" s="11" t="s">
         <v>17</v>
@@ -3888,12 +3894,12 @@
         <v>18</v>
       </c>
       <c r="L58" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>12</v>
@@ -3914,10 +3920,10 @@
         <v>0.13</v>
       </c>
       <c r="H59" s="11" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I59" s="15" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J59" s="11" t="s">
         <v>17</v>
@@ -3926,12 +3932,12 @@
         <v>18</v>
       </c>
       <c r="L59" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>21</v>
@@ -3952,10 +3958,10 @@
         <v>0.125</v>
       </c>
       <c r="H60" s="11" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I60" s="15" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>24</v>
@@ -3964,12 +3970,12 @@
         <v>43</v>
       </c>
       <c r="L60" s="11" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>12</v>
@@ -3978,10 +3984,10 @@
         <v>44.1</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F61" s="1">
         <v>1</v>
@@ -3993,13 +3999,13 @@
         <v>47</v>
       </c>
       <c r="I61" s="15" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J61" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K61" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L61" s="11" t="s">
         <v>18</v>
@@ -4007,7 +4013,7 @@
     </row>
     <row r="62" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>40</v>
@@ -4016,10 +4022,10 @@
         <v>44.1</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F62" s="1">
         <v>1</v>
@@ -4031,7 +4037,7 @@
         <v>47</v>
       </c>
       <c r="I62" s="15" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J62" s="11" t="s">
         <v>26</v>
@@ -4045,7 +4051,7 @@
     </row>
     <row r="63" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>12</v>
@@ -4054,7 +4060,7 @@
         <v>44.1</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>46</v>
@@ -4069,7 +4075,7 @@
         <v>47</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>17</v>
@@ -4083,7 +4089,7 @@
     </row>
     <row r="64" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>40</v>
@@ -4095,7 +4101,7 @@
         <v>30</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F64" s="1">
         <v>1</v>
@@ -4107,21 +4113,21 @@
         <v>32</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K64" s="11" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="L64" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>12</v>
@@ -4133,7 +4139,7 @@
         <v>45</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F65" s="1">
         <v>1</v>
@@ -4142,24 +4148,24 @@
         <v>0.13</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I65" s="15" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>18</v>
       </c>
       <c r="L65" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>12</v>
@@ -4171,7 +4177,7 @@
         <v>45</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F66" s="1">
         <v>1</v>
@@ -4180,16 +4186,16 @@
         <v>0.13</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I66" s="15" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J66" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K66" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L66" s="11" t="s">
         <v>18</v>
@@ -4197,7 +4203,7 @@
     </row>
     <row r="67" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>12</v>
@@ -4209,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F67" s="1">
         <v>1</v>
@@ -4218,24 +4224,24 @@
         <v>0.13</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I67" s="15" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J67" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K67" s="11" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L67" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>12</v>
@@ -4244,10 +4250,10 @@
         <v>93.164999999999992</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F68" s="1">
         <v>1</v>
@@ -4256,24 +4262,24 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H68" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="I68" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="J68" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K68" s="11" t="s">
         <v>300</v>
       </c>
-      <c r="I68" s="15" t="s">
-        <v>301</v>
-      </c>
-      <c r="J68" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K68" s="11" t="s">
-        <v>302</v>
-      </c>
       <c r="L68" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>12</v>
@@ -4282,7 +4288,7 @@
         <v>61.792999999999999</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>46</v>
@@ -4294,10 +4300,10 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H69" s="11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="I69" s="15" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J69" s="11" t="s">
         <v>17</v>
@@ -4311,7 +4317,7 @@
     </row>
     <row r="70" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>12</v>
@@ -4332,10 +4338,10 @@
         <v>0.13</v>
       </c>
       <c r="H70" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I70" s="15" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J70" s="11" t="s">
         <v>17</v>
@@ -4344,12 +4350,12 @@
         <v>18</v>
       </c>
       <c r="L70" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>12</v>
@@ -4358,7 +4364,7 @@
         <v>33.305999999999997</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>14</v>
@@ -4370,10 +4376,10 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H71" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J71" s="11" t="s">
         <v>17</v>
@@ -4382,12 +4388,12 @@
         <v>18</v>
       </c>
       <c r="L71" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>12</v>
@@ -4411,7 +4417,7 @@
         <v>41</v>
       </c>
       <c r="I72" s="15" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>17</v>
@@ -4420,12 +4426,12 @@
         <v>18</v>
       </c>
       <c r="L72" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>12</v>
@@ -4437,7 +4443,7 @@
         <v>51</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F73" s="1">
         <v>1</v>
@@ -4446,10 +4452,10 @@
         <v>0.13</v>
       </c>
       <c r="H73" s="11" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I73" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J73" s="11" t="s">
         <v>18</v>
@@ -4463,7 +4469,7 @@
     </row>
     <row r="74" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>40</v>
@@ -4475,7 +4481,7 @@
         <v>51</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F74" s="1">
         <v>1</v>
@@ -4484,10 +4490,10 @@
         <v>0.11</v>
       </c>
       <c r="H74" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="I74" s="15" t="s">
         <v>309</v>
-      </c>
-      <c r="I74" s="15" t="s">
-        <v>311</v>
       </c>
       <c r="J74" s="11" t="s">
         <v>24</v>
@@ -4501,7 +4507,7 @@
     </row>
     <row r="75" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>12</v>
@@ -4510,10 +4516,10 @@
         <v>51.799499999999995</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F75" s="1">
         <v>1</v>
@@ -4525,21 +4531,21 @@
         <v>47</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K75" s="11" t="s">
         <v>18</v>
       </c>
       <c r="L75" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>12</v>
@@ -4548,7 +4554,7 @@
         <v>50.625</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E76" s="10" t="s">
         <v>14</v>
@@ -4563,7 +4569,7 @@
         <v>47</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>17</v>
@@ -4572,12 +4578,12 @@
         <v>18</v>
       </c>
       <c r="L76" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>12</v>
@@ -4586,10 +4592,10 @@
         <v>58.871999999999993</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F77" s="1">
         <v>1</v>
@@ -4601,13 +4607,13 @@
         <v>47</v>
       </c>
       <c r="I77" s="15" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J77" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K77" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L77" s="11" t="s">
         <v>18</v>
@@ -4615,7 +4621,7 @@
     </row>
     <row r="78" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>12</v>
@@ -4624,10 +4630,10 @@
         <v>58.871999999999993</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F78" s="1">
         <v>1</v>
@@ -4639,7 +4645,7 @@
         <v>47</v>
       </c>
       <c r="I78" s="15" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J78" s="11" t="s">
         <v>17</v>
@@ -4648,12 +4654,12 @@
         <v>18</v>
       </c>
       <c r="L78" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>12</v>
@@ -4674,10 +4680,10 @@
         <v>0.127</v>
       </c>
       <c r="H79" s="11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="I79" s="15" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J79" s="11" t="s">
         <v>17</v>
@@ -4686,12 +4692,12 @@
         <v>18</v>
       </c>
       <c r="L79" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>12</v>
@@ -4703,7 +4709,7 @@
         <v>30</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F80" s="1">
         <v>1</v>
@@ -4712,24 +4718,24 @@
         <v>0.125</v>
       </c>
       <c r="H80" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="I80" s="15" t="s">
         <v>316</v>
       </c>
-      <c r="I80" s="15" t="s">
-        <v>318</v>
-      </c>
       <c r="J80" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K80" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="L80" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>12</v>
@@ -4738,10 +4744,10 @@
         <v>36.799999999999997</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F81" s="1">
         <v>1</v>
@@ -4753,21 +4759,21 @@
         <v>47</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K81" s="11" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="L81" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="82" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>40</v>
@@ -4788,10 +4794,10 @@
         <v>0.12</v>
       </c>
       <c r="H82" s="12" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J82" s="11" t="s">
         <v>26</v>
@@ -4805,10 +4811,10 @@
     </row>
     <row r="83" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C83" s="7">
         <v>43.932000000000002</v>
@@ -4829,7 +4835,7 @@
         <v>22</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J83" s="11" t="s">
         <v>26</v>
@@ -4843,10 +4849,10 @@
     </row>
     <row r="84" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C84" s="7">
         <v>43.932000000000002</v>
@@ -4867,7 +4873,7 @@
         <v>22</v>
       </c>
       <c r="I84" s="15" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J84" s="11" t="s">
         <v>17</v>
@@ -4876,12 +4882,12 @@
         <v>18</v>
       </c>
       <c r="L84" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="85" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>12</v>
@@ -4902,10 +4908,10 @@
         <v>0.13</v>
       </c>
       <c r="H85" s="11" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J85" s="11" t="s">
         <v>17</v>
@@ -4914,12 +4920,12 @@
         <v>18</v>
       </c>
       <c r="L85" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>12</v>
@@ -4943,7 +4949,7 @@
         <v>41</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J86" s="11" t="s">
         <v>17</v>
@@ -4952,12 +4958,12 @@
         <v>18</v>
       </c>
       <c r="L86" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="87" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>12</v>
@@ -4981,7 +4987,7 @@
         <v>41</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J87" s="11" t="s">
         <v>17</v>
@@ -4990,24 +4996,24 @@
         <v>18</v>
       </c>
       <c r="L87" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C88" s="7">
         <v>50.982399999999998</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F88" s="1">
         <v>1</v>
@@ -5016,16 +5022,16 @@
         <v>0.128</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I88" s="15" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J88" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K88" s="11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="L88" s="11" t="s">
         <v>18</v>
@@ -5033,7 +5039,7 @@
     </row>
     <row r="89" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>40</v>
@@ -5042,10 +5048,10 @@
         <v>50.982399999999998</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F89" s="1">
         <v>1</v>
@@ -5054,10 +5060,10 @@
         <v>0.125</v>
       </c>
       <c r="H89" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J89" s="11" t="s">
         <v>24</v>
@@ -5071,7 +5077,7 @@
     </row>
     <row r="90" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>12</v>
@@ -5095,7 +5101,7 @@
         <v>52</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>17</v>
@@ -5104,12 +5110,12 @@
         <v>18</v>
       </c>
       <c r="L90" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>12</v>
@@ -5118,10 +5124,10 @@
         <v>57.874499999999998</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F91" s="1">
         <v>1</v>
@@ -5130,16 +5136,16 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H91" s="11" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="I91" s="15" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J91" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K91" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L91" s="11" t="s">
         <v>18</v>
@@ -5147,7 +5153,7 @@
     </row>
     <row r="92" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>12</v>
@@ -5156,10 +5162,10 @@
         <v>57.874499999999998</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F92" s="1">
         <v>1</v>
@@ -5168,24 +5174,24 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="H92" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="I92" s="15" t="s">
         <v>331</v>
       </c>
-      <c r="I92" s="15" t="s">
-        <v>333</v>
-      </c>
       <c r="J92" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K92" s="11" t="s">
         <v>18</v>
       </c>
       <c r="L92" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>12</v>
@@ -5197,7 +5203,7 @@
         <v>30</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F93" s="1">
         <v>1</v>
@@ -5206,24 +5212,24 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I93" s="15" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K93" s="11" t="s">
         <v>18</v>
       </c>
       <c r="L93" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>12</v>
@@ -5235,7 +5241,7 @@
         <v>30</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F94" s="1">
         <v>1</v>
@@ -5244,24 +5250,24 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I94" s="15" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K94" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="L94" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>12</v>
@@ -5270,10 +5276,10 @@
         <v>60.861599999999996</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F95" s="1">
         <v>1</v>
@@ -5282,24 +5288,24 @@
         <v>0.13</v>
       </c>
       <c r="H95" s="11" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I95" s="15" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J95" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K95" s="11" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L95" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>12</v>
@@ -5308,10 +5314,10 @@
         <v>89.088999999999999</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F96" s="1">
         <v>1</v>
@@ -5320,16 +5326,16 @@
         <v>0.129</v>
       </c>
       <c r="H96" s="11" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="I96" s="15" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J96" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K96" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L96" s="11" t="s">
         <v>18</v>
@@ -5337,7 +5343,7 @@
     </row>
     <row r="97" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>12</v>
@@ -5349,7 +5355,7 @@
         <v>30</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F97" s="1">
         <v>1</v>
@@ -5361,21 +5367,21 @@
         <v>32</v>
       </c>
       <c r="I97" s="15" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J97" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K97" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="L97" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="98" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>12</v>
@@ -5384,10 +5390,10 @@
         <v>94.86</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F98" s="1">
         <v>1</v>
@@ -5396,24 +5402,24 @@
         <v>0.13800000000000001</v>
       </c>
       <c r="H98" s="11" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="I98" s="15" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J98" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K98" s="11" t="s">
         <v>18</v>
       </c>
       <c r="L98" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="99" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>12</v>
@@ -5425,7 +5431,7 @@
         <v>51</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F99" s="1">
         <v>1</v>
@@ -5434,10 +5440,10 @@
         <v>0.13</v>
       </c>
       <c r="H99" s="11" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I99" s="15" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J99" s="11" t="s">
         <v>18</v>
@@ -5451,7 +5457,7 @@
     </row>
     <row r="100" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>12</v>
@@ -5463,7 +5469,7 @@
         <v>51</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F100" s="1">
         <v>1</v>
@@ -5472,10 +5478,10 @@
         <v>0.125</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="I100" s="15" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>18</v>
@@ -5489,7 +5495,7 @@
     </row>
     <row r="101" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>12</v>
@@ -5501,7 +5507,7 @@
         <v>51</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F101" s="1">
         <v>1</v>
@@ -5510,10 +5516,10 @@
         <v>0.12</v>
       </c>
       <c r="H101" s="12" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I101" s="15" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J101" s="11" t="s">
         <v>18</v>
@@ -5527,7 +5533,7 @@
     </row>
     <row r="102" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>21</v>
@@ -5539,7 +5545,7 @@
         <v>51</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F102" s="1">
         <v>1</v>
@@ -5548,10 +5554,10 @@
         <v>0.125</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="I102" s="15" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>18</v>
@@ -5565,7 +5571,7 @@
     </row>
     <row r="103" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>12</v>
@@ -5577,7 +5583,7 @@
         <v>51</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F103" s="1">
         <v>1</v>
@@ -5586,10 +5592,10 @@
         <v>0.13</v>
       </c>
       <c r="H103" s="11" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="I103" s="15" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="J103" s="11" t="s">
         <v>18</v>
@@ -5603,7 +5609,7 @@
     </row>
     <row r="104" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>12</v>
@@ -5615,7 +5621,7 @@
         <v>51</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F104" s="1">
         <v>1</v>
@@ -5624,10 +5630,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H104" s="11" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I104" s="15" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J104" s="11" t="s">
         <v>18</v>
@@ -5641,7 +5647,7 @@
     </row>
     <row r="105" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>12</v>
@@ -5650,10 +5656,10 @@
         <v>59.36</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F105" s="1">
         <v>1</v>
@@ -5662,16 +5668,16 @@
         <v>0.13200000000000001</v>
       </c>
       <c r="H105" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I105" s="15" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="J105" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K105" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L105" s="11" t="s">
         <v>18</v>
@@ -5679,7 +5685,7 @@
     </row>
     <row r="106" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>12</v>
@@ -5688,10 +5694,10 @@
         <v>47.488</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E106" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F106" s="1">
         <v>1</v>
@@ -5700,10 +5706,10 @@
         <v>0.13</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I106" s="15" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>17</v>
@@ -5712,12 +5718,12 @@
         <v>18</v>
       </c>
       <c r="L106" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="107" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>12</v>
@@ -5726,10 +5732,10 @@
         <v>49.896000000000001</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F107" s="1">
         <v>1</v>
@@ -5738,16 +5744,16 @@
         <v>0.13500000000000001</v>
       </c>
       <c r="H107" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I107" s="15" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J107" s="11" t="s">
         <v>17</v>
       </c>
       <c r="K107" s="11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="L107" s="11" t="s">
         <v>18</v>
@@ -5755,7 +5761,7 @@
     </row>
     <row r="108" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>12</v>
@@ -5767,7 +5773,7 @@
         <v>30</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F108" s="1">
         <v>1</v>
@@ -5776,10 +5782,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H108" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I108" s="15" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J108" s="11" t="s">
         <v>17</v>
@@ -5788,12 +5794,12 @@
         <v>18</v>
       </c>
       <c r="L108" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="109" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>40</v>
@@ -5802,7 +5808,7 @@
         <v>63.429599999999994</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>14</v>
@@ -5814,10 +5820,10 @@
         <v>0.125</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I109" s="15" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="J109" s="11" t="s">
         <v>26</v>
@@ -5831,7 +5837,7 @@
     </row>
     <row r="110" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>21</v>
@@ -5840,7 +5846,7 @@
         <v>63.429599999999994</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E110" s="10" t="s">
         <v>14</v>
@@ -5852,10 +5858,10 @@
         <v>0.12</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I110" s="15" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>24</v>
@@ -5864,12 +5870,12 @@
         <v>43</v>
       </c>
       <c r="L110" s="11" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>40</v>
@@ -5878,10 +5884,10 @@
         <v>69.884999999999991</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F111" s="1">
         <v>1</v>
@@ -5893,7 +5899,7 @@
         <v>47</v>
       </c>
       <c r="I111" s="15" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="J111" s="11" t="s">
         <v>24</v>
@@ -5907,7 +5913,7 @@
     </row>
     <row r="112" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>40</v>
@@ -5919,7 +5925,7 @@
         <v>51</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F112" s="1">
         <v>1</v>
@@ -5928,10 +5934,10 @@
         <v>0.12</v>
       </c>
       <c r="H112" s="12" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I112" s="15" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="J112" s="11" t="s">
         <v>24</v>
@@ -5945,7 +5951,7 @@
     </row>
     <row r="113" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A113" s="24" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B113" s="24" t="s">
         <v>12</v>
@@ -5954,10 +5960,10 @@
         <v>69.695999999999998</v>
       </c>
       <c r="D113" s="24" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E113" s="26" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F113" s="27">
         <v>1</v>
@@ -5966,24 +5972,24 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="H113" s="29" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I113" s="30" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="J113" s="29" t="s">
         <v>17</v>
       </c>
       <c r="K113" s="29" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L113" s="29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>12</v>
@@ -5995,7 +6001,7 @@
         <v>51</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F114" s="1">
         <v>4</v>
@@ -6007,13 +6013,13 @@
         <v>52</v>
       </c>
       <c r="I114" s="14" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="J114" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K114" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="L114" s="12" t="s">
         <v>17</v>
@@ -6021,7 +6027,7 @@
     </row>
     <row r="115" spans="1:12" ht="72" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>12</v>
@@ -6030,10 +6036,10 @@
         <v>58.87</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F115" s="1">
         <v>4</v>
@@ -6042,19 +6048,95 @@
         <v>0.13</v>
       </c>
       <c r="H115" s="12" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="I115" s="14" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J115" s="12" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K115" s="12" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="L115" s="12" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C116" s="5">
+        <v>64.819999999999993</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" s="1">
+        <v>4</v>
+      </c>
+      <c r="G116" s="19">
+        <v>0.13</v>
+      </c>
+      <c r="H116" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="I116" s="14" t="s">
+        <v>375</v>
+      </c>
+      <c r="J116" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="K116" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L116" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A117" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C117" s="5">
+        <v>42.78</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" s="1">
+        <v>4</v>
+      </c>
+      <c r="G117" s="17">
+        <v>0.115</v>
+      </c>
+      <c r="H117" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I117" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="J117" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="K117" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L117" s="12" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>